<commit_message>
refine Q3 validation and normalize result workbooks
</commit_message>
<xml_diff>
--- a/src/附件5/result1.xlsx
+++ b/src/附件5/result1.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="0.0000_ "/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,13 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="宋体"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -69,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -94,6 +101,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1964,10 +1972,10 @@
           <t>0:00-4:00</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="10" t="n">
         <v>4500</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <v>0</v>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -1975,7 +1983,7 @@
           <t>0:00</t>
         </is>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="10" t="n">
         <v>6000</v>
       </c>
     </row>
@@ -1985,10 +1993,10 @@
           <t>4:00-8:00</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="10" t="n">
         <v>833.3333333333333</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>5947.419750000019</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1996,7 +2004,7 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="10" t="n">
         <v>6000</v>
       </c>
     </row>
@@ -2006,10 +2014,10 @@
           <t>8:00-12:00</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="10" t="n">
         <v>3954.630954732539</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="10" t="n">
         <v>2121.418433333333</v>
       </c>
     </row>
@@ -2019,10 +2027,10 @@
           <t>12:00-16:00</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="10" t="n">
         <v>6119.368510288064</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <v>91.1013833333335</v>
       </c>
     </row>
@@ -2032,10 +2040,10 @@
           <t>16:00-20:00</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="9" t="n">
+      <c r="B6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>5068.68685</v>
       </c>
     </row>
@@ -2045,10 +2053,10 @@
           <t>20:00-24:00</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>5333.333333333332</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>3571.31315</v>
       </c>
     </row>

</xml_diff>